<commit_message>
Corrected Fransi salary numbers.
</commit_message>
<xml_diff>
--- a/Screw Drivers/Endbericht/Unterlagen/Verwendungsnachweis_ScrewDrivers_1.xlsx
+++ b/Screw Drivers/Endbericht/Unterlagen/Verwendungsnachweis_ScrewDrivers_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\ScrewDriversMFG\Screw Drivers\Endbericht\Unterlagen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62207CBD-A46B-451B-9477-1276264B88FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B1017FA-5609-4EE7-AA8F-A341B832FF6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43350" yWindow="2400" windowWidth="27525" windowHeight="25830" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="47415" yWindow="2100" windowWidth="27525" windowHeight="25830" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quoten" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="230">
   <si>
     <t>Einzelkostenliste – Screw Drivers, Projekt-Nr. G-18/25-1-P</t>
   </si>
@@ -341,18 +341,12 @@
     <t>Brutto 3.504,00 + SV-AG 734.83 + Zus. AG 66.50</t>
   </si>
   <si>
-    <t>C – PERSONALKOSTEN FRANSISKA DAMARA AGUSTINA  (nur ansetzen nach Anzeige gem. AGB C.1)</t>
-  </si>
-  <si>
     <t>Programmierung / QA / Design</t>
   </si>
   <si>
     <t>F. D. Agustina</t>
   </si>
   <si>
-    <t>SCHAETZUNG aus Netto 2.053,49 - durch Lohnjournal ersetzen</t>
-  </si>
-  <si>
     <t>D – OUTSOURCING ART / ANIMATION (Lucas Mößner / Skybound 3D, Mannheim – Kleinunternehmer § 19 UStG)</t>
   </si>
   <si>
@@ -365,18 +359,6 @@
     <t>Rechnung</t>
   </si>
   <si>
-    <t>SB000003</t>
-  </si>
-  <si>
-    <t>28.01.2025</t>
-  </si>
-  <si>
-    <t>01/2025</t>
-  </si>
-  <si>
-    <t>Vorentwicklung – vor Maßnahmebeginn, nicht ansetzbar</t>
-  </si>
-  <si>
     <t>SB000004</t>
   </si>
   <si>
@@ -476,9 +458,6 @@
     <t>12/2025</t>
   </si>
   <si>
-    <t>SB000015</t>
-  </si>
-  <si>
     <t>E – NEBENKOSTEN</t>
   </si>
   <si>
@@ -743,10 +722,10 @@
     <t>Erbrachte Leistung</t>
   </si>
   <si>
-    <t>Muss später ausgezahlt werden</t>
-  </si>
-  <si>
-    <t>Wurde später ausgezahlt</t>
+    <t>C – PERSONALKOSTEN FRANSISKA DAMARA AGUSTINA</t>
+  </si>
+  <si>
+    <t>Brutto 3.000,00 + SV-AG 635.85 + Zus. AG 84.00</t>
   </si>
 </sst>
 </file>
@@ -809,7 +788,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -840,12 +819,6 @@
         <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -874,7 +847,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -902,10 +875,6 @@
     <xf numFmtId="4" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1181,22 +1150,22 @@
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>16</v>
@@ -1205,10 +1174,10 @@
         <v>98</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1223,7 +1192,7 @@
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="2" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1238,7 +1207,7 @@
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="2" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1253,7 +1222,7 @@
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="2" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1268,7 +1237,7 @@
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="2" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1281,7 +1250,7 @@
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
       <c r="E12" s="2" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -1294,7 +1263,7 @@
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="2" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -1307,7 +1276,7 @@
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="2" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -1320,7 +1289,7 @@
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="2" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -1335,7 +1304,7 @@
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="2" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1350,7 +1319,7 @@
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="2" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1365,7 +1334,7 @@
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="2" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1380,7 +1349,7 @@
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="2" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1393,7 +1362,7 @@
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="2" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1406,7 +1375,7 @@
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="2" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1419,7 +1388,7 @@
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
       <c r="E22" s="2" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1432,7 +1401,7 @@
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
       <c r="E23" s="2" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1447,7 +1416,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1462,7 +1431,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1477,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -1488,7 +1457,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1542,10 +1511,10 @@
         <v>9</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="K4" s="6" t="s">
         <v>10</v>
@@ -2393,18 +2362,18 @@
         <v>4000</v>
       </c>
       <c r="J23" s="10">
-        <v>4000</v>
+        <v>3826</v>
       </c>
       <c r="K23" s="11">
         <v>1</v>
       </c>
       <c r="L23" s="10">
         <f t="shared" si="0"/>
-        <v>4000</v>
+        <v>3826</v>
       </c>
       <c r="M23" s="10">
         <f t="shared" si="1"/>
-        <v>4000</v>
+        <v>3826</v>
       </c>
       <c r="N23" s="2" t="s">
         <v>55</v>
@@ -2439,18 +2408,18 @@
         <v>4000</v>
       </c>
       <c r="J24" s="10">
-        <v>4000</v>
+        <v>3524</v>
       </c>
       <c r="K24" s="11">
         <v>1</v>
       </c>
       <c r="L24" s="10">
         <f t="shared" si="0"/>
-        <v>4000</v>
+        <v>3524</v>
       </c>
       <c r="M24" s="10">
         <f t="shared" si="1"/>
-        <v>4000</v>
+        <v>3524</v>
       </c>
       <c r="N24" s="2" t="s">
         <v>55</v>
@@ -2803,7 +2772,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="9">
         <v>27</v>
       </c>
@@ -2850,9 +2819,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>101</v>
+        <v>228</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -2867,23 +2836,17 @@
       <c r="L34" s="8"/>
       <c r="M34" s="8"/>
       <c r="N34" s="8"/>
-      <c r="Q34" s="22">
-        <f>J9-I9+J10-I10+J11-I11+J12-I12+J13-I13</f>
-        <v>22113.200000000001</v>
-      </c>
-      <c r="R34" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="Q34" s="22"/>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="9">
         <v>28</v>
       </c>
       <c r="B35" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="D35" s="9" t="s">
         <v>17</v>
@@ -2901,10 +2864,12 @@
         <v>91</v>
       </c>
       <c r="I35" s="12">
-        <v>3700</v>
+        <f>3000+635.85+84</f>
+        <v>3719.85</v>
       </c>
       <c r="J35" s="12">
-        <v>3700</v>
+        <f>3000+635.85+84</f>
+        <v>3719.85</v>
       </c>
       <c r="K35" s="11">
         <f>Quoten!D25</f>
@@ -2912,28 +2877,25 @@
       </c>
       <c r="L35" s="10">
         <f>J35*K35</f>
-        <v>3700</v>
+        <v>3719.85</v>
       </c>
       <c r="M35" s="10">
         <f>L35</f>
-        <v>3700</v>
+        <v>3719.85</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="R35" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="9">
         <v>29</v>
       </c>
       <c r="B36" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="D36" s="9" t="s">
         <v>17</v>
@@ -2951,10 +2913,12 @@
         <v>95</v>
       </c>
       <c r="I36" s="12">
-        <v>3700</v>
+        <f>3000+635.85+84</f>
+        <v>3719.85</v>
       </c>
       <c r="J36" s="12">
-        <v>3700</v>
+        <f>3000+635.85+84</f>
+        <v>3719.85</v>
       </c>
       <c r="K36" s="11">
         <f>Quoten!D26</f>
@@ -2962,19 +2926,19 @@
       </c>
       <c r="L36" s="10">
         <f>J36*K36</f>
-        <v>3700</v>
+        <v>3719.85</v>
       </c>
       <c r="M36" s="10">
         <f>L36</f>
-        <v>3700</v>
+        <v>3719.85</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -2990,718 +2954,628 @@
       <c r="M37" s="8"/>
       <c r="N37" s="8"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A38" s="23">
-        <v>30</v>
-      </c>
-      <c r="B38" s="23" t="s">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A38" s="9">
+        <v>31</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D38" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C38" s="23" t="s">
+      <c r="E38" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="D38" s="23" t="s">
+      <c r="F38" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="E38" s="23" t="s">
+      <c r="G38" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="F38" s="23" t="s">
+      <c r="H38" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="I38" s="10">
+        <v>2415</v>
+      </c>
+      <c r="J38" s="10">
+        <v>2415</v>
+      </c>
+      <c r="K38" s="11">
+        <v>1</v>
+      </c>
+      <c r="L38" s="10">
+        <f t="shared" ref="L38:L48" si="4">J38*K38</f>
+        <v>2415</v>
+      </c>
+      <c r="M38" s="10">
+        <f t="shared" ref="M38:M48" si="5">L38</f>
+        <v>2415</v>
+      </c>
+      <c r="N38" s="2"/>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A39" s="9">
+        <v>32</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="E39" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="G38" s="23" t="s">
+      <c r="F39" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="H38" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="I38" s="24">
-        <v>1215</v>
-      </c>
-      <c r="J38" s="24">
-        <v>1215</v>
-      </c>
-      <c r="K38" s="25">
-        <v>0</v>
-      </c>
-      <c r="L38" s="24">
-        <f t="shared" ref="L38:L50" si="4">J38*K38</f>
-        <v>0</v>
-      </c>
-      <c r="M38" s="24">
-        <f t="shared" ref="M38:M50" si="5">L38</f>
-        <v>0</v>
-      </c>
-      <c r="N38" s="26" t="s">
+      <c r="G39" s="9" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A39" s="9">
-        <v>31</v>
-      </c>
-      <c r="B39" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D39" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="E39" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="F39" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="G39" s="9" t="s">
-        <v>115</v>
-      </c>
       <c r="H39" s="9" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="I39" s="10">
-        <v>2415</v>
+        <v>2040</v>
       </c>
       <c r="J39" s="10">
-        <v>2415</v>
+        <v>2040</v>
       </c>
       <c r="K39" s="11">
         <v>1</v>
       </c>
       <c r="L39" s="10">
         <f t="shared" si="4"/>
-        <v>2415</v>
+        <v>2040</v>
       </c>
       <c r="M39" s="10">
         <f t="shared" si="5"/>
-        <v>2415</v>
+        <v>2040</v>
       </c>
       <c r="N39" s="2"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="9">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B40" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D40" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C40" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>108</v>
-      </c>
       <c r="E40" s="9" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I40" s="10">
-        <v>2040</v>
+        <v>1440</v>
       </c>
       <c r="J40" s="10">
-        <v>2040</v>
+        <v>1440</v>
       </c>
       <c r="K40" s="11">
         <v>1</v>
       </c>
       <c r="L40" s="10">
         <f t="shared" si="4"/>
-        <v>2040</v>
+        <v>1440</v>
       </c>
       <c r="M40" s="10">
         <f t="shared" si="5"/>
-        <v>2040</v>
+        <v>1440</v>
       </c>
       <c r="N40" s="2"/>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="9">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B41" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D41" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C41" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D41" s="9" t="s">
-        <v>108</v>
-      </c>
       <c r="E41" s="9" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="I41" s="10">
-        <v>1440</v>
+        <v>2130</v>
       </c>
       <c r="J41" s="10">
-        <v>1440</v>
+        <v>2130</v>
       </c>
       <c r="K41" s="11">
         <v>1</v>
       </c>
       <c r="L41" s="10">
         <f t="shared" si="4"/>
-        <v>1440</v>
+        <v>2130</v>
       </c>
       <c r="M41" s="10">
         <f t="shared" si="5"/>
-        <v>1440</v>
+        <v>2130</v>
       </c>
       <c r="N41" s="2"/>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="9">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B42" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D42" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C42" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>108</v>
-      </c>
       <c r="E42" s="9" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="I42" s="10">
-        <v>2130</v>
+        <v>1170</v>
       </c>
       <c r="J42" s="10">
-        <v>2130</v>
+        <v>1170</v>
       </c>
       <c r="K42" s="11">
         <v>1</v>
       </c>
       <c r="L42" s="10">
         <f t="shared" si="4"/>
-        <v>2130</v>
+        <v>1170</v>
       </c>
       <c r="M42" s="10">
         <f t="shared" si="5"/>
-        <v>2130</v>
+        <v>1170</v>
       </c>
       <c r="N42" s="2"/>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="9">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B43" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D43" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C43" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>108</v>
-      </c>
       <c r="E43" s="9" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="H43" s="9" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I43" s="10">
-        <v>1170</v>
+        <v>1185</v>
       </c>
       <c r="J43" s="10">
-        <v>1170</v>
+        <v>1185</v>
       </c>
       <c r="K43" s="11">
         <v>1</v>
       </c>
       <c r="L43" s="10">
         <f t="shared" si="4"/>
-        <v>1170</v>
+        <v>1185</v>
       </c>
       <c r="M43" s="10">
         <f t="shared" si="5"/>
-        <v>1170</v>
+        <v>1185</v>
       </c>
       <c r="N43" s="2"/>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" s="9">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B44" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D44" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C44" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>108</v>
-      </c>
       <c r="E44" s="9" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I44" s="10">
-        <v>1185</v>
+        <v>1290</v>
       </c>
       <c r="J44" s="10">
-        <v>1185</v>
+        <v>1290</v>
       </c>
       <c r="K44" s="11">
         <v>1</v>
       </c>
       <c r="L44" s="10">
         <f t="shared" si="4"/>
-        <v>1185</v>
+        <v>1290</v>
       </c>
       <c r="M44" s="10">
         <f t="shared" si="5"/>
-        <v>1185</v>
+        <v>1290</v>
       </c>
       <c r="N44" s="2"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="9">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B45" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D45" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C45" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D45" s="9" t="s">
-        <v>108</v>
-      </c>
       <c r="E45" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="H45" s="9" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I45" s="10">
-        <v>1290</v>
+        <v>1800</v>
       </c>
       <c r="J45" s="10">
-        <v>1290</v>
+        <v>1800</v>
       </c>
       <c r="K45" s="11">
         <v>1</v>
       </c>
       <c r="L45" s="10">
         <f t="shared" si="4"/>
-        <v>1290</v>
+        <v>1800</v>
       </c>
       <c r="M45" s="10">
         <f t="shared" si="5"/>
-        <v>1290</v>
+        <v>1800</v>
       </c>
       <c r="N45" s="2"/>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="9">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B46" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D46" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C46" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D46" s="9" t="s">
-        <v>108</v>
-      </c>
       <c r="E46" s="9" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="I46" s="10">
-        <v>1800</v>
+        <v>2870</v>
       </c>
       <c r="J46" s="10">
-        <v>1800</v>
+        <v>2870</v>
       </c>
       <c r="K46" s="11">
         <v>1</v>
       </c>
       <c r="L46" s="10">
         <f t="shared" si="4"/>
-        <v>1800</v>
+        <v>2870</v>
       </c>
       <c r="M46" s="10">
         <f t="shared" si="5"/>
-        <v>1800</v>
+        <v>2870</v>
       </c>
       <c r="N46" s="2"/>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="9">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B47" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D47" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C47" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D47" s="9" t="s">
-        <v>108</v>
-      </c>
       <c r="E47" s="9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="H47" s="9" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="I47" s="10">
-        <v>2870</v>
+        <v>2835</v>
       </c>
       <c r="J47" s="10">
-        <v>2870</v>
+        <v>2835</v>
       </c>
       <c r="K47" s="11">
         <v>1</v>
       </c>
       <c r="L47" s="10">
         <f t="shared" si="4"/>
-        <v>2870</v>
+        <v>2835</v>
       </c>
       <c r="M47" s="10">
         <f t="shared" si="5"/>
-        <v>2870</v>
+        <v>2835</v>
       </c>
       <c r="N47" s="2"/>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="9">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B48" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D48" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C48" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D48" s="9" t="s">
-        <v>108</v>
-      </c>
       <c r="E48" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I48" s="10">
-        <v>2835</v>
+        <v>2425</v>
       </c>
       <c r="J48" s="10">
-        <v>2835</v>
+        <v>2425</v>
       </c>
       <c r="K48" s="11">
         <v>1</v>
       </c>
       <c r="L48" s="10">
         <f t="shared" si="4"/>
-        <v>2835</v>
+        <v>2425</v>
       </c>
       <c r="M48" s="10">
         <f t="shared" si="5"/>
-        <v>2835</v>
+        <v>2425</v>
       </c>
       <c r="N48" s="2"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A49" s="9">
-        <v>41</v>
-      </c>
-      <c r="B49" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C49" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D49" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="E49" s="9" t="s">
+      <c r="A49" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B49" s="8"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="8"/>
+      <c r="F49" s="8"/>
+      <c r="G49" s="8"/>
+      <c r="H49" s="8"/>
+      <c r="I49" s="8"/>
+      <c r="J49" s="8"/>
+      <c r="K49" s="8"/>
+      <c r="L49" s="8"/>
+      <c r="M49" s="8"/>
+      <c r="N49" s="8"/>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A50" s="9">
+        <v>43</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="D50" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="F49" s="9" t="s">
+      <c r="E50" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="F50" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="H49" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="I49" s="10">
-        <v>2425</v>
-      </c>
-      <c r="J49" s="10">
-        <v>2425</v>
-      </c>
-      <c r="K49" s="11">
-        <v>1</v>
-      </c>
-      <c r="L49" s="10">
-        <f t="shared" si="4"/>
-        <v>2425</v>
-      </c>
-      <c r="M49" s="10">
-        <f t="shared" si="5"/>
-        <v>2425</v>
-      </c>
-      <c r="N49" s="2"/>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A50" s="23">
-        <v>42</v>
-      </c>
-      <c r="B50" s="23" t="s">
-        <v>106</v>
-      </c>
-      <c r="C50" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="D50" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="E50" s="23" t="s">
+      <c r="G50" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="F50" s="23" t="s">
-        <v>144</v>
-      </c>
-      <c r="G50" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="H50" s="23" t="s">
-        <v>144</v>
-      </c>
-      <c r="I50" s="24">
-        <v>375</v>
-      </c>
-      <c r="J50" s="24">
-        <v>375</v>
-      </c>
-      <c r="K50" s="25">
+      <c r="H50" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="I50" s="10">
+        <v>2032.25</v>
+      </c>
+      <c r="J50" s="10">
+        <v>2032.25</v>
+      </c>
+      <c r="K50" s="11">
+        <v>1</v>
+      </c>
+      <c r="L50" s="10">
+        <f>J50*K50</f>
+        <v>2032.25</v>
+      </c>
+      <c r="M50" s="10">
         <v>0</v>
       </c>
-      <c r="L50" s="24">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="M50" s="24">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="N50" s="26"/>
+      <c r="N50" s="2" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A51" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="B51" s="8"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="8"/>
-      <c r="F51" s="8"/>
-      <c r="G51" s="8"/>
-      <c r="H51" s="8"/>
-      <c r="I51" s="8"/>
-      <c r="J51" s="8"/>
-      <c r="K51" s="8"/>
-      <c r="L51" s="8"/>
-      <c r="M51" s="8"/>
-      <c r="N51" s="8"/>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A52" s="9">
-        <v>43</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="C52" s="9" t="s">
+      <c r="A51" s="9">
+        <v>44</v>
+      </c>
+      <c r="B51" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="D52" s="9" t="s">
+      <c r="C51" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="E52" s="9" t="s">
+      <c r="D51" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="F52" s="9" t="s">
+      <c r="E51" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="G52" s="9" t="s">
+      <c r="F51" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="G51" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="H52" s="9" t="s">
+      <c r="H51" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="I51" s="10">
+        <v>4391.1000000000004</v>
+      </c>
+      <c r="J51" s="10">
+        <v>4391.1000000000004</v>
+      </c>
+      <c r="K51" s="11">
+        <v>1</v>
+      </c>
+      <c r="L51" s="10">
+        <f>J51*K51</f>
+        <v>4391.1000000000004</v>
+      </c>
+      <c r="M51" s="10">
+        <f>L51</f>
+        <v>4391.1000000000004</v>
+      </c>
+      <c r="N51" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="I52" s="10">
-        <v>2032.25</v>
-      </c>
-      <c r="J52" s="10">
-        <v>2032.25</v>
-      </c>
-      <c r="K52" s="11">
-        <v>1</v>
-      </c>
-      <c r="L52" s="10">
-        <f>J52*K52</f>
-        <v>2032.25</v>
-      </c>
-      <c r="M52" s="10">
-        <v>0</v>
-      </c>
-      <c r="N52" s="2" t="s">
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A53" s="8"/>
+      <c r="B53" s="7" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A53" s="9">
-        <v>44</v>
-      </c>
-      <c r="B53" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="C53" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="D53" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="E53" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="F53" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="G53" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="H53" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="I53" s="10">
-        <v>4391.1000000000004</v>
-      </c>
-      <c r="J53" s="10">
-        <v>4391.1000000000004</v>
-      </c>
-      <c r="K53" s="11">
-        <v>1</v>
-      </c>
-      <c r="L53" s="10">
-        <f>J53*K53</f>
-        <v>4391.1000000000004</v>
-      </c>
-      <c r="M53" s="10">
-        <f>L53</f>
-        <v>4391.1000000000004</v>
-      </c>
-      <c r="N53" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A55" s="8"/>
-      <c r="B55" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="C55" s="8"/>
-      <c r="D55" s="8"/>
-      <c r="E55" s="8"/>
-      <c r="F55" s="8"/>
-      <c r="G55" s="8"/>
-      <c r="H55" s="8"/>
-      <c r="I55" s="13">
-        <f>SUM(I5:I53)</f>
-        <v>160480.49000000002</v>
-      </c>
-      <c r="J55" s="13">
-        <f>SUM(J5:J53)</f>
-        <v>149429.65</v>
-      </c>
-      <c r="K55" s="8"/>
-      <c r="L55" s="13">
-        <f>SUM(L5:L53)</f>
-        <v>147839.65</v>
-      </c>
-      <c r="M55" s="13">
-        <f>SUM(M5:M53)</f>
-        <v>145807.4</v>
-      </c>
-      <c r="N55" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="8"/>
+      <c r="F53" s="8"/>
+      <c r="G53" s="8"/>
+      <c r="H53" s="8"/>
+      <c r="I53" s="13">
+        <f>SUM(I5:I51)</f>
+        <v>158930.19000000003</v>
+      </c>
+      <c r="J53" s="13">
+        <f>SUM(J5:J51)</f>
+        <v>147229.35</v>
+      </c>
+      <c r="K53" s="8"/>
+      <c r="L53" s="13">
+        <f>SUM(L5:L51)</f>
+        <v>147229.35</v>
+      </c>
+      <c r="M53" s="13">
+        <f>SUM(M5:M51)</f>
+        <v>145197.1</v>
+      </c>
+      <c r="N53" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3722,38 +3596,38 @@
   <sheetData>
     <row r="1" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15"/>
       <c r="B5" s="15" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -3806,7 +3680,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B8" s="5">
         <v>0.6</v>
@@ -3830,7 +3704,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -3838,8 +3712,8 @@
         <v>16</v>
       </c>
       <c r="B11" s="10">
-        <f>SUMIF(Einzelkostenliste!$C$5:$C$53,"Simon Blasen",Einzelkostenliste!$L$5:$L$53)</f>
-        <v>78429.399999999994</v>
+        <f>SUMIF(Einzelkostenliste!$C$5:$C$51,"Simon Blasen",Einzelkostenliste!$L$5:$L$51)</f>
+        <v>77779.399999999994</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -3847,22 +3721,22 @@
         <v>98</v>
       </c>
       <c r="B12" s="10">
-        <f>SUMIF(Einzelkostenliste!$C$5:$C$53,"Marc Bendt",Einzelkostenliste!$L$5:$L$53)</f>
+        <f>SUMIF(Einzelkostenliste!$C$5:$C$51,"Marc Bendt",Einzelkostenliste!$L$5:$L$51)</f>
         <v>33986.9</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B13" s="10">
-        <f>SUMIF(Einzelkostenliste!$C$5:$C$53,"F. D. Agustina",Einzelkostenliste!$L$5:$L$53)</f>
-        <v>7400</v>
+        <f>SUMIF(Einzelkostenliste!$C$5:$C$51,"F. D. Agustina",Einzelkostenliste!$L$5:$L$51)</f>
+        <v>7439.7</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3870,37 +3744,37 @@
         <v>3</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="B17" s="10">
         <v>50220</v>
       </c>
       <c r="C17" s="10">
         <f>$B$11*B$6+$B$12*B$7+$B$13*B$8</f>
-        <v>59340.579999999994</v>
+        <v>58909.399999999994</v>
       </c>
       <c r="D17" s="10">
         <f t="shared" ref="D17:D22" si="0">MIN(B17,C17)</f>
@@ -3920,19 +3794,19 @@
       </c>
       <c r="H17" s="10">
         <f t="shared" ref="H17:H22" si="4">MAX(0,C17-B17)</f>
-        <v>9120.5799999999945</v>
+        <v>8689.3999999999942</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B18" s="10">
         <v>12600</v>
       </c>
       <c r="C18" s="10">
         <f>$B$11*D$6+$B$12*D$7+$B$13*D$8</f>
-        <v>14857.539999999999</v>
+        <v>14829.009999999998</v>
       </c>
       <c r="D18" s="10">
         <f t="shared" si="0"/>
@@ -3952,12 +3826,12 @@
       </c>
       <c r="H18" s="10">
         <f t="shared" si="4"/>
-        <v>2257.5399999999991</v>
+        <v>2229.0099999999984</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="B19" s="10">
         <v>7560</v>
@@ -3989,14 +3863,14 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B20" s="10">
         <v>25200</v>
       </c>
       <c r="C20" s="10">
         <f>$B$11*F$6+$B$12*F$7+$B$13*F$8</f>
-        <v>28755.735000000001</v>
+        <v>28702.645</v>
       </c>
       <c r="D20" s="10">
         <f t="shared" si="0"/>
@@ -4016,35 +3890,35 @@
       </c>
       <c r="H20" s="10">
         <f t="shared" si="4"/>
-        <v>3555.7350000000006</v>
+        <v>3502.6450000000004</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="B21" s="10">
         <v>11880</v>
       </c>
       <c r="C21" s="10">
         <f>$B$11*C$6+$B$12*C$7+$B$13*C$8</f>
-        <v>11764.409999999998</v>
+        <v>11666.909999999998</v>
       </c>
       <c r="D21" s="10">
         <f t="shared" si="0"/>
-        <v>11764.409999999998</v>
+        <v>11666.909999999998</v>
       </c>
       <c r="E21" s="10">
         <f t="shared" si="1"/>
-        <v>-115.59000000000196</v>
+        <v>-213.09000000000196</v>
       </c>
       <c r="F21" s="18">
         <f t="shared" si="2"/>
-        <v>-9.7297979797981455E-3</v>
+        <v>-1.7936868686868852E-2</v>
       </c>
       <c r="G21" s="10">
         <f t="shared" si="3"/>
-        <v>115.59000000000196</v>
+        <v>213.09000000000196</v>
       </c>
       <c r="H21" s="10">
         <f t="shared" si="4"/>
@@ -4053,13 +3927,13 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="B22" s="10">
         <v>21600</v>
       </c>
       <c r="C22" s="10">
-        <f>SUMIF(Einzelkostenliste!$C$5:$C$53,"Lucas Mößner (Skybound 3D)",Einzelkostenliste!$L$5:$L$53)</f>
+        <f>SUMIF(Einzelkostenliste!$C$5:$C$51,"Lucas Mößner (Skybound 3D)",Einzelkostenliste!$L$5:$L$51)</f>
         <v>21600</v>
       </c>
       <c r="D22" s="10">
@@ -4085,7 +3959,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B23" s="13">
         <f>SUM(B17:B22)</f>
@@ -4093,46 +3967,46 @@
       </c>
       <c r="C23" s="13">
         <f>SUM(C17:C22)</f>
-        <v>141416.29999999999</v>
+        <v>140806</v>
       </c>
       <c r="D23" s="13">
         <f>SUM(D17:D22)</f>
-        <v>126482.44500000001</v>
+        <v>126384.94500000001</v>
       </c>
       <c r="E23" s="13">
         <f>SUM(E17:E22)</f>
-        <v>-2577.5550000000021</v>
+        <v>-2675.0550000000021</v>
       </c>
       <c r="F23" s="19">
         <f t="shared" si="2"/>
-        <v>-1.9971757322175748E-2</v>
+        <v>-2.0727219897722006E-2</v>
       </c>
       <c r="G23" s="13">
         <f>SUM(G17:G22)</f>
-        <v>2577.5550000000021</v>
+        <v>2675.0550000000021</v>
       </c>
       <c r="H23" s="13">
         <f>SUM(H17:H22)</f>
-        <v>14933.854999999994</v>
+        <v>14421.054999999993</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="H24" s="20">
         <f>H23</f>
-        <v>14933.854999999994</v>
+        <v>14421.054999999993</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="B26" s="10">
         <v>4391.1000000000004</v>
@@ -4151,7 +4025,7 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="B27" s="10">
         <v>2032.25</v>
@@ -4169,7 +4043,7 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="B28" s="13">
         <f>SUM(B26:B27)</f>
@@ -4190,7 +4064,7 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="B30" s="13">
         <f>B23+B28</f>
@@ -4198,40 +4072,40 @@
       </c>
       <c r="C30" s="13">
         <f>C23+C28</f>
-        <v>147839.65</v>
+        <v>147229.35</v>
       </c>
       <c r="D30" s="13">
         <f>D23+D28</f>
-        <v>132905.79500000001</v>
+        <v>132808.29500000001</v>
       </c>
       <c r="E30" s="13">
         <f>E23+E28</f>
-        <v>-2577.5550000000021</v>
+        <v>-2675.0550000000021</v>
       </c>
       <c r="F30" s="19">
         <f>IFERROR(E30/B30,0)</f>
-        <v>-1.9024883869493942E-2</v>
+        <v>-1.9744529493845569E-2</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="B32" s="10">
         <v>133451.1</v>
       </c>
       <c r="D32" s="21">
         <f>D23+D26</f>
-        <v>130873.54500000001</v>
+        <v>130776.04500000001</v>
       </c>
       <c r="E32" s="21">
         <f>D32-B32</f>
-        <v>-2577.554999999993</v>
+        <v>-2675.054999999993</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -4253,21 +4127,21 @@
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>13</v>
@@ -4275,26 +4149,26 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="B5" s="10">
         <v>67741.679999999993</v>
       </c>
       <c r="C5" s="10">
         <f>MIN(67741.68,Schlusskostenstand!D30*0.5)</f>
-        <v>66452.897500000006</v>
+        <v>66404.147500000006</v>
       </c>
       <c r="D5" s="10">
         <f>C5-B5</f>
-        <v>-1288.7824999999866</v>
+        <v>-1337.5324999999866</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="B6" s="10">
         <v>54666.64</v>
@@ -4307,31 +4181,31 @@
         <v>2.0000000004074536E-2</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="B7" s="10">
         <v>13075.03</v>
       </c>
       <c r="C7" s="10">
         <f>Schlusskostenstand!D30-C5-C6</f>
-        <v>11786.237500000003</v>
+        <v>11737.487500000003</v>
       </c>
       <c r="D7" s="10">
         <f>C7-B7</f>
-        <v>-1288.7924999999977</v>
+        <v>-1337.5424999999977</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="B8" s="13">
         <f>SUM(B5:B7)</f>
@@ -4339,44 +4213,44 @@
       </c>
       <c r="C8" s="13">
         <f>SUM(C5:C7)</f>
-        <v>132905.79500000001</v>
+        <v>132808.29500000001</v>
       </c>
       <c r="D8" s="13">
         <f>SUM(D5:D7)</f>
-        <v>-2577.5549999999803</v>
+        <v>-2675.0549999999803</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="C9" s="21">
         <f>C8-Schlusskostenstand!D30</f>
         <v>0</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B13" s="10">
         <v>33870.839999999997</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B14" s="10">
         <v>27096.67</v>
@@ -4385,7 +4259,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B15" s="10">
         <f>SUM(B13:B14)</f>
@@ -4394,14 +4268,14 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B16" s="13">
         <f>C5-B15</f>
-        <v>5485.3875000000116</v>
+        <v>5436.6375000000116</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>